<commit_message>
ajustando nome de concept
</commit_message>
<xml_diff>
--- a/SCRTheoryCodeBook.xlsx
+++ b/SCRTheoryCodeBook.xlsx
@@ -190,7 +190,7 @@
     <t>Avoiding system obsolescence</t>
   </si>
   <si>
-    <t>Preventing System Obsolescence</t>
+    <t>System Obsolescence</t>
   </si>
   <si>
     <t>06-interview-translation.docx</t>
@@ -2217,10 +2217,10 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -3087,7 +3087,7 @@
       <c r="C27" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="D27" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E27" s="3" t="s">
@@ -3107,7 +3107,7 @@
       <c r="C28" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E28" s="3" t="s">
@@ -3127,7 +3127,7 @@
       <c r="C29" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E29" s="3" t="s">
@@ -3147,7 +3147,7 @@
       <c r="C30" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E30" s="3" t="s">
@@ -3167,7 +3167,7 @@
       <c r="C31" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E31" s="3" t="s">
@@ -3187,7 +3187,7 @@
       <c r="C32" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E32" s="3" t="s">
@@ -3207,7 +3207,7 @@
       <c r="C33" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E33" s="3" t="s">
@@ -3227,7 +3227,7 @@
       <c r="C34" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="D34" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E34" s="3" t="s">
@@ -3247,7 +3247,7 @@
       <c r="C35" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D35" s="3" t="s">
+      <c r="D35" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E35" s="3" t="s">
@@ -3267,7 +3267,7 @@
       <c r="C36" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D36" s="3" t="s">
+      <c r="D36" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E36" s="3" t="s">
@@ -3287,7 +3287,7 @@
       <c r="C37" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D37" s="3" t="s">
+      <c r="D37" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E37" s="3" t="s">
@@ -3307,7 +3307,7 @@
       <c r="C38" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D38" s="3" t="s">
+      <c r="D38" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E38" s="3" t="s">
@@ -3327,7 +3327,7 @@
       <c r="C39" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D39" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E39" s="3" t="s">
@@ -3347,7 +3347,7 @@
       <c r="C40" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D40" s="3" t="s">
+      <c r="D40" s="4" t="s">
         <v>53</v>
       </c>
       <c r="E40" s="3" t="s">
@@ -16327,7 +16327,7 @@
       <c r="C689" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D689" s="4" t="s">
+      <c r="D689" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E689" s="2" t="s">
@@ -16367,7 +16367,7 @@
       <c r="C690" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D690" s="4" t="s">
+      <c r="D690" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E690" s="2" t="s">
@@ -16407,7 +16407,7 @@
       <c r="C691" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D691" s="4" t="s">
+      <c r="D691" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E691" s="2" t="s">
@@ -16447,7 +16447,7 @@
       <c r="C692" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D692" s="4" t="s">
+      <c r="D692" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E692" s="2" t="s">
@@ -16487,7 +16487,7 @@
       <c r="C693" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D693" s="4" t="s">
+      <c r="D693" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E693" s="2" t="s">
@@ -16527,7 +16527,7 @@
       <c r="C694" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D694" s="4" t="s">
+      <c r="D694" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E694" s="2" t="s">
@@ -16567,7 +16567,7 @@
       <c r="C695" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D695" s="4" t="s">
+      <c r="D695" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E695" s="2" t="s">
@@ -16607,7 +16607,7 @@
       <c r="C696" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D696" s="4" t="s">
+      <c r="D696" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E696" s="2" t="s">
@@ -16647,7 +16647,7 @@
       <c r="C697" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D697" s="4" t="s">
+      <c r="D697" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E697" s="2" t="s">
@@ -16687,7 +16687,7 @@
       <c r="C698" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D698" s="4" t="s">
+      <c r="D698" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E698" s="2" t="s">
@@ -16727,7 +16727,7 @@
       <c r="C699" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D699" s="4" t="s">
+      <c r="D699" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E699" s="2" t="s">
@@ -16767,7 +16767,7 @@
       <c r="C700" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D700" s="4" t="s">
+      <c r="D700" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E700" s="2" t="s">
@@ -16807,7 +16807,7 @@
       <c r="C701" s="2" t="s">
         <v>584</v>
       </c>
-      <c r="D701" s="4" t="s">
+      <c r="D701" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E701" s="2" t="s">
@@ -16847,7 +16847,7 @@
       <c r="C702" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D702" s="4" t="s">
+      <c r="D702" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E702" s="2" t="s">
@@ -16887,7 +16887,7 @@
       <c r="C703" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D703" s="4" t="s">
+      <c r="D703" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E703" s="2" t="s">
@@ -16927,7 +16927,7 @@
       <c r="C704" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D704" s="4" t="s">
+      <c r="D704" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E704" s="2" t="s">
@@ -16967,7 +16967,7 @@
       <c r="C705" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D705" s="4" t="s">
+      <c r="D705" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E705" s="2" t="s">
@@ -17007,7 +17007,7 @@
       <c r="C706" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D706" s="4" t="s">
+      <c r="D706" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E706" s="2" t="s">
@@ -17047,7 +17047,7 @@
       <c r="C707" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D707" s="4" t="s">
+      <c r="D707" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E707" s="2" t="s">
@@ -17087,7 +17087,7 @@
       <c r="C708" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D708" s="4" t="s">
+      <c r="D708" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E708" s="2" t="s">
@@ -17127,7 +17127,7 @@
       <c r="C709" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D709" s="4" t="s">
+      <c r="D709" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E709" s="2" t="s">
@@ -17167,7 +17167,7 @@
       <c r="C710" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D710" s="4" t="s">
+      <c r="D710" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E710" s="2" t="s">
@@ -17207,7 +17207,7 @@
       <c r="C711" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D711" s="4" t="s">
+      <c r="D711" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E711" s="2" t="s">
@@ -17247,7 +17247,7 @@
       <c r="C712" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D712" s="4" t="s">
+      <c r="D712" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E712" s="2" t="s">
@@ -17287,7 +17287,7 @@
       <c r="C713" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D713" s="4" t="s">
+      <c r="D713" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E713" s="2" t="s">
@@ -17327,7 +17327,7 @@
       <c r="C714" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D714" s="4" t="s">
+      <c r="D714" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E714" s="2" t="s">
@@ -17367,7 +17367,7 @@
       <c r="C715" s="2" t="s">
         <v>595</v>
       </c>
-      <c r="D715" s="4" t="s">
+      <c r="D715" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E715" s="2" t="s">
@@ -17407,7 +17407,7 @@
       <c r="C716" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="D716" s="4" t="s">
+      <c r="D716" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E716" s="2" t="s">
@@ -17447,7 +17447,7 @@
       <c r="C717" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="D717" s="4" t="s">
+      <c r="D717" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E717" s="2" t="s">
@@ -17487,7 +17487,7 @@
       <c r="C718" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="D718" s="4" t="s">
+      <c r="D718" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E718" s="2" t="s">
@@ -17527,7 +17527,7 @@
       <c r="C719" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="D719" s="4" t="s">
+      <c r="D719" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E719" s="2" t="s">
@@ -17567,7 +17567,7 @@
       <c r="C720" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="D720" s="4" t="s">
+      <c r="D720" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E720" s="2" t="s">
@@ -17607,7 +17607,7 @@
       <c r="C721" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="D721" s="4" t="s">
+      <c r="D721" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E721" s="2" t="s">
@@ -17647,7 +17647,7 @@
       <c r="C722" s="2" t="s">
         <v>606</v>
       </c>
-      <c r="D722" s="4" t="s">
+      <c r="D722" s="5" t="s">
         <v>585</v>
       </c>
       <c r="E722" s="2" t="s">
@@ -17687,7 +17687,7 @@
       <c r="C723" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D723" s="4" t="s">
+      <c r="D723" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E723" s="2" t="s">
@@ -17727,7 +17727,7 @@
       <c r="C724" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D724" s="4" t="s">
+      <c r="D724" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E724" s="2" t="s">
@@ -17767,7 +17767,7 @@
       <c r="C725" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D725" s="4" t="s">
+      <c r="D725" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E725" s="2" t="s">
@@ -17807,7 +17807,7 @@
       <c r="C726" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D726" s="4" t="s">
+      <c r="D726" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E726" s="2" t="s">
@@ -17847,7 +17847,7 @@
       <c r="C727" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D727" s="4" t="s">
+      <c r="D727" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E727" s="2" t="s">
@@ -17887,7 +17887,7 @@
       <c r="C728" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D728" s="4" t="s">
+      <c r="D728" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E728" s="2" t="s">
@@ -17927,7 +17927,7 @@
       <c r="C729" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D729" s="4" t="s">
+      <c r="D729" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E729" s="2" t="s">
@@ -17967,7 +17967,7 @@
       <c r="C730" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D730" s="4" t="s">
+      <c r="D730" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E730" s="2" t="s">
@@ -18007,7 +18007,7 @@
       <c r="C731" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D731" s="4" t="s">
+      <c r="D731" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E731" s="2" t="s">
@@ -18047,7 +18047,7 @@
       <c r="C732" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D732" s="4" t="s">
+      <c r="D732" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E732" s="2" t="s">
@@ -18087,7 +18087,7 @@
       <c r="C733" s="2" t="s">
         <v>610</v>
       </c>
-      <c r="D733" s="4" t="s">
+      <c r="D733" s="5" t="s">
         <v>596</v>
       </c>
       <c r="E733" s="2" t="s">
@@ -18127,10 +18127,10 @@
       <c r="C734" s="3" t="s">
         <v>621</v>
       </c>
-      <c r="D734" s="5" t="s">
+      <c r="D734" s="4" t="s">
         <v>622</v>
       </c>
-      <c r="E734" s="5" t="s">
+      <c r="E734" s="4" t="s">
         <v>623</v>
       </c>
       <c r="F734" s="3" t="s">
@@ -18147,10 +18147,10 @@
       <c r="C735" s="3" t="s">
         <v>625</v>
       </c>
-      <c r="D735" s="5" t="s">
+      <c r="D735" s="4" t="s">
         <v>622</v>
       </c>
-      <c r="E735" s="5" t="s">
+      <c r="E735" s="4" t="s">
         <v>623</v>
       </c>
       <c r="F735" s="3" t="s">
@@ -18167,10 +18167,10 @@
       <c r="C736" s="3" t="s">
         <v>625</v>
       </c>
-      <c r="D736" s="5" t="s">
+      <c r="D736" s="4" t="s">
         <v>622</v>
       </c>
-      <c r="E736" s="5" t="s">
+      <c r="E736" s="4" t="s">
         <v>623</v>
       </c>
       <c r="F736" s="3" t="s">
@@ -18619,16 +18619,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="7" t="s">

</xml_diff>

<commit_message>
atualizando data avaliability para versao final
</commit_message>
<xml_diff>
--- a/SCRTheoryCodeBook.xlsx
+++ b/SCRTheoryCodeBook.xlsx
@@ -8,14 +8,14 @@
   </sheets>
   <definedNames>
     <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">FullCodeBook!$A$1:$Z$954</definedName>
-    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Six Cs Structure'!$A$1:$E$75</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'Six Cs Structure'!$A$1:$E$76</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4717" uniqueCount="629">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4799" uniqueCount="640">
   <si>
     <t>Document</t>
   </si>
@@ -2088,6 +2088,39 @@
   </si>
   <si>
     <t>video.js Since Video.js components are now un-transpiled ES6 classes `extend()` needs to be able to handle them since `videojs.extend(videojs.getComponent('Component') {...})` is the most common usecase for this method. This string check is apparently the only way to detect ES6 classes. It isn't future proof and supposedly will not work on some older platforms but that is likely not a huge concern since we are 1) dropping support for most older platforms and 2) deprecating this method and encouraging the use of native classes instead.</t>
+  </si>
+  <si>
+    <t>[Speaker 2]  So, for example, have you ever used it to give you code recommendations? I gave you an example in our conversation about Java 8 and Java 17, for example. For example, Arrow Functions in JavaScript.  Have you ever used a more traditional code, an older way of seeing it? In the CHATGPT, how can I transform this into a Arrow Function? Is it in this mode that you use? Can you explain how you use this for your code?  [Speaker 1]  It's pretty much in this line, using JavaScript as an example. In React, I started developing the project and it was still done with classes. And then you had to bind everything, it was a totally different structure. And then came a version of React 9, I confess I don't remember which one it was. But they introduced Arrow Functions, everything became hooks in the system, everything became a function. And then I had to do this process of putting a part of the code, it wasn't everything. I usually took specific parts of the code to understand what was different, and from there I replicated it in other places. So it was more of a way to understand the changes between the versions, and from there I did the migration. I didn't use it as a migration tool, that is, I didn't put all the code there, it migrated and I copied it. It was more of a way to understand the specificities of each version.</t>
+  </si>
+  <si>
+    <t>LLM-based support for source code rejuvenation</t>
+  </si>
+  <si>
+    <t>[Speaker 2]  And you've already touched on the subject, right? In your opinion, what is the impact of LMMs, of artificial intelligence, for this question of code evolution? How do you see this?  [Speaker 1]  Let's go. Let's play statistics now, okay? Let's go.  Statistics are talking about what is normal. Normal is the average, right? Most of the AI today, it was trained with mass.  Mass is the normal down. Because we know that quality is not the preference of most developers. In fact, it's just delivering.  So, I think ok, I think it's cool who uses it, to a certain extent. Why? Because if you want to stay mediocre, you will always use it for everything.  If you know how to use it and get the best out of it, no. You can really take advantage of it. You go to work on Junior, for example, and you have to improve the code all the time.  Very few times will you have a really good code coming out of the AI. And that's why I made my own improvisations, I've already made several codes, right? But nowadays, apart from Sonnet, which is fucking good, the worst part is to stay there in the mediocre.  Sonnet goes to the reasonable sometimes. It's good for you to do CSS, because it's something trivial, everything has to be done. It's good for you to do a simple front-end thing.  But when you're going to work with complex things, man, most of the time it's going to suck. In addition to a big point that people don't realize. When you put code there and it's not business, you're taking a little problem, a chance of failing your code.  Because it's used to train.</t>
+  </si>
+  <si>
+    <t>Exactly. But, in short, AI is good, but it has to evolve a lot. And Junior shouldn't use it.  I've seen a lot of Junior who doesn't know how to code anymore.  [Speaker 2]  So your recommendation, for example, your vision, is that it has to be used with caution. For example, a Junior could use it to learn about a new feature, about the type, instead of taking a code from that system and asking it to implement such a thing. What do you think about GitHub's Copilot?  [Speaker 1]  I know people today who have a middle developer, who think it's a senior developer, and they can't do the minimum without Copilot. So, how do we do it? The guy thinks it's senior developer, because he can do some things full of broken bugs.  And in this same project, who was carrying it was Junior. It's complicated. It's complicated, right?  AI is a very annoying theme in this aspect, because it gets into the hype, and the hype is often not the best. I don't know if you've worked with a lot of different people, a lot of projects, but what do you see? The level was already bad, it's just getting worse.  You're seeing worse and worse things. Imagine, for me, AI is like Stack Overflow, but faster. If you took a Stack Overflow code, threw it in your code and it worked, it could work.  Many times it didn't work. It's the same thing, but it's an improved Stack Overflow. That's it.  But it's going to normal, man. 99% of the applications you're going to work on will work. You're going to work with something that needs performance and something that's good or to last, no.  But most of the time, what's going to happen? If the guy delivered in that development environment, there's a little bit of data, it's something very calm, something good, it's going to work. In a few months, a few weeks, or even when the production goes up soon, it's going to go bad and you're going to have to patch it up.</t>
+  </si>
+  <si>
+    <t>Hmm. So, interesting, man. In that respect, I think it has something to do with the AI itself, right?  AI is something very interesting, but I think it's starting to get better now, for training itself, right? With DeepSeek and so on, right? There are new hardwares that are coming out now to make it cheaper to train, but there's a big deficiency in something specific.  Most of it is generic. And generic things, they will never reach the same performance as something that is specialized in itself. So, if you research this aspect of AI and make improvements in code and evolution of the language, cool, but specify a language first.  In this case, too. Don't try to do something generic and make an upgrade, because the chance of failure will be great.</t>
+  </si>
+  <si>
+    <t>At the moment I'm not using it in any way. And at work, I particularly don't know anyone who uses it, no. At least not that they speak openly about using it.  [Speaker 1]  Do you think it would be a problem, for example, within the company you work for, to use an LLM to support you in implementation?  [Speaker 2]  Well, the code and bank data are confidential, so I think there may be a privacy problem with regards to the data, since all these LLMs collect it. So I think there could be a problem, yes.</t>
+  </si>
+  <si>
+    <t>Man, to create new code, I've used it a lot. Not only IDE, but nowadays Copilot, or any model of artificial intelligence, this is being used routinely, by all the team developers. But to refactor code, as I said, we will revisit the code, we don't use a lot of tools.  We get suggestions on how to improve performance, but I'm still very fond of legibility, and nowadays the code created, either by IA or IDE, we still need to improve it, to make it a little more legible, a little more like us, you know?</t>
+  </si>
+  <si>
+    <t>Man, it's interesting. I would give it a chance. I'm still a little behind with this.  I think it's a very ready-made solution, I'm still a little behind, but I still believe a lot in the potential. Despite being behind, I totally support and support this type of innovation, because, man, Copilot came out of it, and today everyone uses Copilot independently. There's another lib called CLINE, which I use as a plugin in VS Code.  It reads all your folders, all your passes, it asks for permission to read everything, and with this context it gives you more... It's a little more precise when it comes to creating and refactoring the code. So there are, yes, I believe the model can evolve to the point of doing this.  But for legacy code, I haven't used this yet, refactoring, getting the code. What I did a lot was get a code that was all confused, legacy, throw it in LLM and say, tell me what it means, so I can understand, to know what's going on there. And of course, with suggestions for improvement, with suggestions to update the code, I don't think I've ever done it.  Like, update this code for me.</t>
+  </si>
+  <si>
+    <t>Yes, maybe because of my age, I'm a little older, I'm almost 40, 37. So I'm used to breaking my head. That's the standard I knew.  But the youngest people on the team, I see that they trust it totally. Like, go there, create it, do it. And there's no problem.  I'm the one who's more likely to use it and still have the human intervention in this type of coding.</t>
+  </si>
+  <si>
+    <t>Dude, the impact is being absurd. In short, I'll explain this better. But in short, a developer who uses LLMs to develop produces the equivalent of three developers without LLMs. Like, in terms of functionality, amount of code, quality of code. So today the impact is, we need fewer developers to do the same amount as they do. What would you do with two, three? In our team, it was like that. The amount of tickets solved with LLM increased the speed a lot.</t>
+  </si>
+  <si>
+    <t>Let me think here. About... To conclude, I would like to address the use of LLMs and the generational trends that are currently popular and widely discussed.  I feel that the quality of the code is improving. The quality of test creation is also improving. Just to complement what I was saying before.  Today, automated tests, integration tests, the whole process of running the pipeline, checking if there is any error. All this structural part of the business is making it a lot easier, the LLM. So, the question of thinking about the business, the developer is no longer doing a lot of manual work.  He's being more of a consultant, a consultant of... I understand what you want to do. I know the technologies you need to do this.  And the whole process is being... The LLM is being used as a bed for the developer to go there and just punctually do the things that are needed in this process. Nowadays...  I'll give you an example. I don't see myself as an infrastructure guy anymore. Because today the cloud does everything.  It's like an AWS of life. I click a button and it does everything. So nowadays, there's no guy who goes there and configures everything for us and for everything to work.  And that's how it's working for all the processes of code development. Both deploy, construction, environment creation, creation of everything, we're using a more automated process. Test creation, integration, anyway.  in conclusion, we, as developers, at least me, as a developer and our team, we work more punctually on the intelligence part of the business. How can we do this in an optimized way? Because doing it manually, the LLM does it, but in an intelligent way, it still needs the developer.  And I think that's the differential. We're evolving for this. We're not going to be replaced.  We're just going to use the tools we have in a better way.</t>
   </si>
   <si>
     <t>Occurences by Code</t>
@@ -18177,19 +18210,266 @@
         <v>476</v>
       </c>
     </row>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1">
+      <c r="A737" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B737" s="4" t="s">
+        <v>627</v>
+      </c>
+      <c r="C737" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D737" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E737" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F737" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="738" ht="15.75" customHeight="1">
+      <c r="A738" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B738" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="C738" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D738" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E738" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F738" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="739" ht="15.75" customHeight="1">
+      <c r="A739" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B739" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="C739" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D739" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E739" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F739" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="740" ht="15.75" customHeight="1">
+      <c r="A740" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B740" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="C740" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D740" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E740" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F740" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="741" ht="15.75" customHeight="1">
+      <c r="A741" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B741" s="4" t="s">
+        <v>630</v>
+      </c>
+      <c r="C741" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D741" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E741" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F741" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="742" ht="15.75" customHeight="1">
+      <c r="A742" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B742" s="4" t="s">
+        <v>631</v>
+      </c>
+      <c r="C742" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D742" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E742" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F742" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="743" ht="15.75" customHeight="1">
+      <c r="A743" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B743" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="C743" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D743" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E743" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F743" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="744" ht="15.75" customHeight="1">
+      <c r="A744" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B744" s="4" t="s">
+        <v>632</v>
+      </c>
+      <c r="C744" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D744" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E744" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F744" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="745" ht="15.75" customHeight="1">
+      <c r="A745" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B745" s="4" t="s">
+        <v>633</v>
+      </c>
+      <c r="C745" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D745" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E745" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F745" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="746" ht="15.75" customHeight="1">
+      <c r="A746" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B746" s="4" t="s">
+        <v>634</v>
+      </c>
+      <c r="C746" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D746" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E746" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F746" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="747" ht="15.75" customHeight="1">
+      <c r="A747" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B747" s="4" t="s">
+        <v>635</v>
+      </c>
+      <c r="C747" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D747" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E747" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F747" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="748" ht="15.75" customHeight="1">
+      <c r="A748" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B748" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="C748" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D748" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E748" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F748" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="749" ht="15.75" customHeight="1">
+      <c r="A749" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B749" s="4" t="s">
+        <v>637</v>
+      </c>
+      <c r="C749" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="D749" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="E749" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="F749" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
     <row r="750" ht="15.75" customHeight="1"/>
     <row r="751" ht="15.75" customHeight="1"/>
     <row r="752" ht="15.75" customHeight="1"/>
@@ -18632,7 +18912,7 @@
         <v>5</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>627</v>
+        <v>638</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -19808,7 +20088,7 @@
     </row>
     <row r="34">
       <c r="A34" s="15" t="s">
-        <v>628</v>
+        <v>639</v>
       </c>
       <c r="B34" s="12" t="s">
         <v>258</v>
@@ -21247,20 +21527,20 @@
       <c r="X73" s="2"/>
     </row>
     <row r="74">
-      <c r="A74" s="33" t="s">
-        <v>625</v>
-      </c>
-      <c r="B74" s="34" t="s">
-        <v>622</v>
-      </c>
-      <c r="C74" s="34" t="s">
-        <v>623</v>
-      </c>
-      <c r="D74" s="34" t="s">
+      <c r="A74" s="20" t="s">
+        <v>628</v>
+      </c>
+      <c r="B74" s="20" t="s">
+        <v>596</v>
+      </c>
+      <c r="C74" s="20" t="s">
+        <v>586</v>
+      </c>
+      <c r="D74" s="20" t="s">
         <v>476</v>
       </c>
-      <c r="E74" s="7">
-        <v>2.0</v>
+      <c r="E74" s="5">
+        <v>11.0</v>
       </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
@@ -21284,7 +21564,7 @@
     </row>
     <row r="75">
       <c r="A75" s="33" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="B75" s="34" t="s">
         <v>622</v>
@@ -21296,7 +21576,7 @@
         <v>476</v>
       </c>
       <c r="E75" s="7">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
@@ -21319,11 +21599,21 @@
       <c r="X75" s="2"/>
     </row>
     <row r="76">
-      <c r="A76" s="2"/>
-      <c r="B76" s="2"/>
-      <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
+      <c r="A76" s="33" t="s">
+        <v>621</v>
+      </c>
+      <c r="B76" s="34" t="s">
+        <v>622</v>
+      </c>
+      <c r="C76" s="34" t="s">
+        <v>623</v>
+      </c>
+      <c r="D76" s="34" t="s">
+        <v>476</v>
+      </c>
+      <c r="E76" s="7">
+        <v>1.0</v>
+      </c>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
@@ -44251,12 +44541,12 @@
       <c r="X957" s="2"/>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$E$75">
-    <sortState ref="A1:E75">
-      <sortCondition ref="D1:D75"/>
-      <sortCondition ref="B1:B75"/>
-      <sortCondition descending="1" ref="E1:E75"/>
-      <sortCondition ref="C1:C75"/>
+  <autoFilter ref="$A$1:$E$76">
+    <sortState ref="A1:E76">
+      <sortCondition ref="D1:D76"/>
+      <sortCondition ref="B1:B76"/>
+      <sortCondition descending="1" ref="E1:E76"/>
+      <sortCondition ref="C1:C76"/>
     </sortState>
   </autoFilter>
   <drawing r:id="rId1"/>

</xml_diff>